<commit_message>
Drop 0 configuration inputs workbook in the guided design: Start here index of the register items by due date and fill-in order, self-contained template sheets with guide band and drop-downs, clearly titled reference sheets, reference lists and questions sheet; closure summary text and the list of legacy record statuses mapped to Data Migration
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/06_BIBS_Templates_BRD-03_Configuration_Inputs_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/06_BIBS_Templates_BRD-03_Configuration_Inputs_v2.0.xlsx
@@ -2299,7 +2299,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="29" customHeight="1">
+    <row r="18" ht="16" customHeight="1">
       <c r="A18" s="9" t="n">
         <v>4</v>
       </c>
@@ -2388,7 +2388,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="120" customHeight="1">
+    <row r="23" ht="95" customHeight="1">
       <c r="A23" s="12" t="n">
         <v>1</v>
       </c>
@@ -2446,7 +2446,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="69" customHeight="1">
+    <row r="24" ht="56" customHeight="1">
       <c r="A24" s="17" t="n">
         <v>2</v>
       </c>
@@ -2504,7 +2504,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="56" customHeight="1">
+    <row r="25" ht="43" customHeight="1">
       <c r="A25" s="12" t="n">
         <v>3</v>
       </c>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="69" customHeight="1">
+    <row r="27" ht="56" customHeight="1">
       <c r="A27" s="12" t="n">
         <v>5</v>
       </c>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="56" customHeight="1">
+    <row r="28" ht="43" customHeight="1">
       <c r="A28" s="17" t="n">
         <v>6</v>
       </c>
@@ -2736,7 +2736,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
+    <row r="29" ht="43" customHeight="1">
       <c r="A29" s="12" t="n">
         <v>7</v>
       </c>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="95" customHeight="1">
+    <row r="30" ht="82" customHeight="1">
       <c r="A30" s="17" t="n">
         <v>8</v>
       </c>
@@ -2852,7 +2852,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="82" customHeight="1">
+    <row r="31" ht="56" customHeight="1">
       <c r="A31" s="12" t="n">
         <v>9</v>
       </c>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="82" customHeight="1">
+    <row r="32" ht="56" customHeight="1">
       <c r="A32" s="17" t="n">
         <v>10</v>
       </c>
@@ -3539,7 +3539,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="47" t="inlineStr">
         <is>
           <t>Example – overwrite or delete</t>
@@ -12640,7 +12640,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="165.5" customHeight="1">
+    <row r="5" ht="115.5" customHeight="1">
       <c r="A5" s="41" t="inlineStr">
         <is>
           <t>Yes or no (YES_NO)</t>
@@ -12684,7 +12684,7 @@
       </c>
       <c r="E6" s="19" t="n"/>
     </row>
-    <row r="7" ht="40.5" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="57" t="inlineStr">
         <is>
           <t>Market segment (MARKET_SEGMENT)</t>
@@ -12756,7 +12756,7 @@
       </c>
       <c r="E10" s="14" t="n"/>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11">
       <c r="A11" s="57" t="n"/>
       <c r="B11" s="14" t="n"/>
       <c r="C11" s="58" t="inlineStr">
@@ -12771,7 +12771,7 @@
       </c>
       <c r="E11" s="14" t="n"/>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12">
       <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Placement after (PLACEMENT_GATE)</t>
@@ -12809,7 +12809,7 @@
       </c>
       <c r="E13" s="19" t="n"/>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14">
       <c r="A14" s="57" t="inlineStr">
         <is>
           <t>TSU review (TSU_REVIEW)</t>
@@ -12915,7 +12915,7 @@
       </c>
       <c r="E19" s="19" t="n"/>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="57" t="inlineStr">
         <is>
           <t>Document type (DOCUMENT_TYPE)</t>
@@ -13137,7 +13137,7 @@
       </c>
       <c r="E33" s="14" t="n"/>
     </row>
-    <row r="34" ht="28" customHeight="1">
+    <row r="34">
       <c r="A34" s="57" t="n"/>
       <c r="B34" s="14" t="n"/>
       <c r="C34" s="58" t="inlineStr">
@@ -13632,7 +13632,7 @@
       </c>
       <c r="E66" s="14" t="n"/>
     </row>
-    <row r="67" ht="28" customHeight="1">
+    <row r="67">
       <c r="A67" s="57" t="n"/>
       <c r="B67" s="14" t="n"/>
       <c r="C67" s="58" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="E71" s="14" t="n"/>
     </row>
-    <row r="72" ht="28" customHeight="1">
+    <row r="72">
       <c r="A72" s="57" t="n"/>
       <c r="B72" s="14" t="n"/>
       <c r="C72" s="58" t="inlineStr">
@@ -13767,7 +13767,7 @@
       </c>
       <c r="E75" s="14" t="n"/>
     </row>
-    <row r="76" ht="28" customHeight="1">
+    <row r="76">
       <c r="A76" s="57" t="n"/>
       <c r="B76" s="14" t="n"/>
       <c r="C76" s="58" t="inlineStr">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="E80" s="14" t="n"/>
     </row>
-    <row r="81" ht="40.5" customHeight="1">
+    <row r="81" ht="28" customHeight="1">
       <c r="A81" s="41" t="inlineStr">
         <is>
           <t>Clause kind (CLAUSE_KIND)</t>
@@ -13967,7 +13967,7 @@
       </c>
       <c r="E87" s="14" t="n"/>
     </row>
-    <row r="88" ht="28" customHeight="1">
+    <row r="88">
       <c r="A88" s="41" t="inlineStr">
         <is>
           <t>Package map action (MAP_ACTION)</t>
@@ -13990,7 +13990,7 @@
       </c>
       <c r="E88" s="19" t="n"/>
     </row>
-    <row r="89" ht="28" customHeight="1">
+    <row r="89">
       <c r="A89" s="41" t="n"/>
       <c r="B89" s="19" t="n"/>
       <c r="C89" s="56" t="inlineStr">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="E95" s="14" t="n"/>
     </row>
-    <row r="96" ht="40.5" customHeight="1">
+    <row r="96" ht="28" customHeight="1">
       <c r="A96" s="41" t="inlineStr">
         <is>
           <t>Product Maintenance list or parameter (PM_LIST_OR_PARAMETER)</t>
@@ -14156,7 +14156,7 @@
       </c>
       <c r="E98" s="19" t="n"/>
     </row>
-    <row r="99" ht="28" customHeight="1">
+    <row r="99">
       <c r="A99" s="41" t="n"/>
       <c r="B99" s="19" t="n"/>
       <c r="C99" s="56" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="E109" s="19" t="n"/>
     </row>
-    <row r="110" ht="40.5" customHeight="1">
+    <row r="110" ht="28" customHeight="1">
       <c r="A110" s="41" t="n"/>
       <c r="B110" s="19" t="n"/>
       <c r="C110" s="56" t="inlineStr">
@@ -14366,7 +14366,7 @@
       </c>
       <c r="E112" s="19" t="n"/>
     </row>
-    <row r="113" ht="28" customHeight="1">
+    <row r="113">
       <c r="A113" s="41" t="n"/>
       <c r="B113" s="19" t="n"/>
       <c r="C113" s="56" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="E114" s="19" t="n"/>
     </row>
-    <row r="115" ht="28" customHeight="1">
+    <row r="115">
       <c r="A115" s="41" t="n"/>
       <c r="B115" s="19" t="n"/>
       <c r="C115" s="56" t="inlineStr">
@@ -14411,7 +14411,7 @@
       </c>
       <c r="E115" s="19" t="n"/>
     </row>
-    <row r="116" ht="28" customHeight="1">
+    <row r="116">
       <c r="A116" s="41" t="n"/>
       <c r="B116" s="19" t="n"/>
       <c r="C116" s="56" t="inlineStr">
@@ -14441,7 +14441,7 @@
       </c>
       <c r="E117" s="19" t="n"/>
     </row>
-    <row r="118" ht="40.5" customHeight="1">
+    <row r="118" ht="28" customHeight="1">
       <c r="A118" s="41" t="n"/>
       <c r="B118" s="19" t="n"/>
       <c r="C118" s="56" t="inlineStr">
@@ -14456,7 +14456,7 @@
       </c>
       <c r="E118" s="19" t="n"/>
     </row>
-    <row r="119" ht="40.5" customHeight="1">
+    <row r="119" ht="28" customHeight="1">
       <c r="A119" s="57" t="inlineStr">
         <is>
           <t>Incentive type (INCENTIVE_TYPE)</t>
@@ -14572,7 +14572,7 @@
       <c r="D126" s="19" t="n"/>
       <c r="E126" s="19" t="n"/>
     </row>
-    <row r="127" ht="28" customHeight="1">
+    <row r="127">
       <c r="A127" s="41" t="n"/>
       <c r="B127" s="19" t="n"/>
       <c r="C127" s="56" t="inlineStr">
@@ -14594,7 +14594,7 @@
       <c r="D128" s="19" t="n"/>
       <c r="E128" s="19" t="n"/>
     </row>
-    <row r="129" ht="40.5" customHeight="1">
+    <row r="129" ht="28" customHeight="1">
       <c r="A129" s="41" t="n"/>
       <c r="B129" s="19" t="n"/>
       <c r="C129" s="56" t="inlineStr">
@@ -14605,7 +14605,7 @@
       <c r="D129" s="19" t="n"/>
       <c r="E129" s="19" t="n"/>
     </row>
-    <row r="130" ht="28" customHeight="1">
+    <row r="130">
       <c r="A130" s="41" t="n"/>
       <c r="B130" s="19" t="n"/>
       <c r="C130" s="56" t="inlineStr">
@@ -14627,7 +14627,7 @@
       <c r="D131" s="19" t="n"/>
       <c r="E131" s="19" t="n"/>
     </row>
-    <row r="132" ht="28" customHeight="1">
+    <row r="132">
       <c r="A132" s="57" t="inlineStr">
         <is>
           <t>Question status (QUESTION_STATUS)</t>
@@ -16251,7 +16251,7 @@
         </is>
       </c>
     </row>
-    <row r="6" outlineLevel="1" ht="28" customHeight="1">
+    <row r="6" outlineLevel="1" ht="15.5" customHeight="1">
       <c r="A6" s="30" t="inlineStr">
         <is>
           <t>How it is loaded</t>
@@ -42116,7 +42116,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="47" t="inlineStr">
         <is>
           <t>Example – overwrite or delete</t>
@@ -51079,7 +51079,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="47" t="inlineStr">
         <is>
           <t>Example – overwrite or delete</t>

</xml_diff>